<commit_message>
Acesso professor e mais features
</commit_message>
<xml_diff>
--- a/planilha importacao.xlsx
+++ b/planilha importacao.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\Documents\GitHub\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\Documents\GitHub\jogo_jornada_conhecimento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E4927C89-ED41-4992-911E-EBAD02BC7BBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E0EB51-FA5A-4465-903B-4EB508C8938F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CA651793-5F75-4CBB-A8B0-B1FD7573FF6D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>id</t>
   </si>
@@ -77,36 +77,35 @@
     <t>tempoLimite</t>
   </si>
   <si>
-    <t>TESTE PERGUNTA IMPORTAÇÃO</t>
-  </si>
-  <si>
-    <t>A</t>
+    <t>Qual a soma de 2+ 2</t>
   </si>
   <si>
     <t>B</t>
   </si>
   <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>D</t>
-  </si>
-  <si>
-    <t>TESTE</t>
-  </si>
-  <si>
-    <t>facil</t>
-  </si>
-  <si>
-    <t>teste</t>
+    <t>matematica</t>
+  </si>
+  <si>
+    <t>Facil</t>
+  </si>
+  <si>
+    <t>Soma de 2+2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -136,7 +135,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -471,7 +470,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0DCF540-779A-47C6-9B7D-C470E4F24736}">
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
@@ -479,14 +478,14 @@
     <col min="3" max="5" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -524,43 +523,41 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s">
-        <v>13</v>
-      </c>
-      <c r="D2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>16</v>
+      <c r="C2">
+        <v>6</v>
+      </c>
+      <c r="D2">
+        <v>4</v>
+      </c>
+      <c r="E2">
+        <v>8</v>
+      </c>
+      <c r="F2">
+        <v>10</v>
       </c>
       <c r="G2" t="s">
         <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="I2" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J2" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="K2">
-        <v>1000</v>
+        <v>100</v>
       </c>
       <c r="L2">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="C12" s="1"/>
+        <v>5</v>
+      </c>
+      <c r="M2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
Implementa IA pra gerar perguntas
</commit_message>
<xml_diff>
--- a/planilha importacao.xlsx
+++ b/planilha importacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\Documents\GitHub\jogo_jornada_conhecimento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E0EB51-FA5A-4465-903B-4EB508C8938F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB2ECD3-89D9-47B5-9EDF-B066B0CD4125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CA651793-5F75-4CBB-A8B0-B1FD7573FF6D}"/>
   </bookViews>
@@ -77,35 +77,27 @@
     <t>tempoLimite</t>
   </si>
   <si>
-    <t>Qual a soma de 2+ 2</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
     <t>matematica</t>
   </si>
   <si>
     <t>Facil</t>
   </si>
   <si>
-    <t>Soma de 2+2</t>
+    <t>Qual é a soma de 10 + 10</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>Soma 10 + 10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -133,9 +125,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -470,7 +461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0DCF540-779A-47C6-9B7D-C470E4F24736}">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
@@ -485,7 +476,7 @@
     <col min="12" max="12" width="11.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -523,41 +514,40 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>20</v>
+      </c>
+      <c r="D2">
+        <v>40</v>
+      </c>
+      <c r="E2">
+        <v>60</v>
+      </c>
+      <c r="F2">
+        <v>80</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
         <v>12</v>
       </c>
-      <c r="C2">
-        <v>6</v>
-      </c>
-      <c r="D2">
-        <v>4</v>
-      </c>
-      <c r="E2">
-        <v>8</v>
-      </c>
-      <c r="F2">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="I2" t="s">
         <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>15</v>
       </c>
       <c r="J2" t="s">
         <v>16</v>
       </c>
       <c r="K2">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="L2">
-        <v>5</v>
-      </c>
-      <c r="M2" s="1"/>
+        <v>30</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>

</xml_diff>

<commit_message>
implementação de botão para baixar planilha modelo
</commit_message>
<xml_diff>
--- a/planilha importacao.xlsx
+++ b/planilha importacao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\natha\Documents\GitHub\jogo_jornada_conhecimento\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB2ECD3-89D9-47B5-9EDF-B066B0CD4125}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1409A66D-610E-474A-91CA-D4E854CB18EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CA651793-5F75-4CBB-A8B0-B1FD7573FF6D}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>id</t>
   </si>
@@ -75,21 +75,6 @@
   </si>
   <si>
     <t>tempoLimite</t>
-  </si>
-  <si>
-    <t>matematica</t>
-  </si>
-  <si>
-    <t>Facil</t>
-  </si>
-  <si>
-    <t>Qual é a soma de 10 + 10</t>
-  </si>
-  <si>
-    <t>A</t>
-  </si>
-  <si>
-    <t>Soma 10 + 10</t>
   </si>
 </sst>
 </file>
@@ -461,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0DCF540-779A-47C6-9B7D-C470E4F24736}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" bestFit="1" customWidth="1"/>
@@ -514,41 +499,6 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2">
-        <v>20</v>
-      </c>
-      <c r="D2">
-        <v>40</v>
-      </c>
-      <c r="E2">
-        <v>60</v>
-      </c>
-      <c r="F2">
-        <v>80</v>
-      </c>
-      <c r="G2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2">
-        <v>150</v>
-      </c>
-      <c r="L2">
-        <v>30</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>